<commit_message>
Build contract-review-flagger skill: SKILL.md, rubric, scripts, entity list, open items
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012r6bKnXcJp9a2cyYVk4obL
</commit_message>
<xml_diff>
--- a/skills/contract-review-flagger/examples/Contract_Review_ESG.xlsx
+++ b/skills/contract-review-flagger/examples/Contract_Review_ESG.xlsx
@@ -1948,7 +1948,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Check 9</t>
+          <t>Check 11</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Annex A, D, E, F are icons only; 7.3 cites wrong annex letters (E and F for D and E).</t>
+          <t>Annex A, D, E, F are icons only; their content is not in the copy (pp. 13, 16-18).</t>
         </is>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Two clauses numbered 7.2; Module 2 annex letters wrong.</t>
+          <t>7.3 Module 2 cites Annex E and F for the attendance and survey templates; they are Annex D and E (pp. 6, 16-17).</t>
         </is>
       </c>
     </row>

</xml_diff>